<commit_message>
modified the project to reduce errors
</commit_message>
<xml_diff>
--- a/Datasets/Q1.xlsx
+++ b/Datasets/Q1.xlsx
@@ -1,134 +1,59 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Avi\HR\New Assignment may 2024\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAA34D60-7CD9-401C-ADC8-C071AA6E3A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="qEaLtqRQ1MZQE7H003s85u8W2GoYx3ACWL7TsTvR2BQ="/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
-  <si>
-    <t>SKU</t>
-  </si>
-  <si>
-    <t>Dimentions ( L X B X H) Inches</t>
-  </si>
-  <si>
-    <t>Weight ( Pounds)</t>
-  </si>
-  <si>
-    <t>MH-107</t>
-  </si>
-  <si>
-    <t>20.5 X 20.5 X 7</t>
-  </si>
-  <si>
-    <t>MH-901</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 X 18.5 X 6.25 </t>
-  </si>
-  <si>
-    <t>MH-805</t>
-  </si>
-  <si>
-    <t>23 X 22.75 X 4.75</t>
-  </si>
-  <si>
-    <t>MH-11500</t>
-  </si>
-  <si>
-    <t>18 X 81 X 14.5</t>
-  </si>
-  <si>
-    <t>Expenses involved in selling</t>
-  </si>
-  <si>
-    <t>Channel Commison</t>
-  </si>
-  <si>
-    <t>Storage (Needs to be calculated for 3 month)</t>
-  </si>
-  <si>
-    <t>2$ Per Cubic Meter per month</t>
-  </si>
-  <si>
-    <t>Clossing fee per order</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5$ for order value below 120$ and 10$ for orders above 120$ </t>
-  </si>
-  <si>
-    <t>Returns</t>
-  </si>
-  <si>
-    <t>10% of revenue</t>
-  </si>
-  <si>
-    <t>Selling price</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="5">
     <font>
+      <name val="Aptos Narrow"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
     </font>
     <font>
-      <strike/>
+      <name val="Aptos Narrow"/>
+      <strike val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -222,156 +147,164 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="18">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="3152775" cy="1409700"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3769613" y="3075150"/>
-          <a:ext cx="3152775" cy="1409700"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cap="flat" cmpd="sng">
-          <a:solidFill>
-            <a:srgbClr val="BABABA"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:round/>
-          <a:headEnd type="none" w="sm" len="sm"/>
-          <a:tailEnd type="none" w="sm" len="sm"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="45700" rIns="91425" bIns="45700" anchor="t" anchorCtr="0">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buNone/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-              <a:sym typeface="Arial"/>
-            </a:rPr>
-            <a:t>Calculate the buying</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-              <a:sym typeface="Arial"/>
-            </a:rPr>
-            <a:t> price of the SKU if we are selling these SKUs with Net margin of 15% </a:t>
-          </a:r>
-          <a:endParaRPr sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -571,124 +504,168 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1000"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="53.5703125" customWidth="1"/>
-    <col min="3" max="3" width="27.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
-    <col min="5" max="26" width="8.5703125" customWidth="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="53.5703125" customWidth="1" min="2" max="2"/>
+    <col width="27.7109375" customWidth="1" min="3" max="3"/>
+    <col width="16.140625" customWidth="1" min="4" max="4"/>
+    <col width="8.5703125" customWidth="1" min="5" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Selling price</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Dimensions ( L X B X H) Inches</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Weight ( Pounds)</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5">
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>MH-107</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="6">
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>20.5 X 20.5 X 7</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="5">
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>MH-901</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
         <v>150</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="6">
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 X 18.5 X 6.25 </t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
         <v>20.5</v>
       </c>
-      <c r="E3" s="7"/>
+      <c r="E3" s="7" t="n"/>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="5">
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MH-805</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
         <v>20.5</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>23 X 22.75 X 4.75</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n">
         <v>14.5</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="9">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>MH-11500</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
         <v>163</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="10">
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>18 X 81 X 14.5</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="15"/>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Expenses involved in selling</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n"/>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="11">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Channel Commison</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
         <v>0.15</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>14</v>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Storage (Needs to be calculated for 3 month)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2$ Per Cubic Meter per month</t>
+        </is>
       </c>
     </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>16</v>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Clossing fee per order</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5$ for order value below 120$ and 10$ for orders above 120$ </t>
+        </is>
       </c>
     </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>18</v>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Returns</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>10% of revenue</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1677,6 +1654,5 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>